<commit_message>
feat: agregar paginación y mejoras en la interfaz de cliente y migración
</commit_message>
<xml_diff>
--- a/backend/uploads/data.xlsx
+++ b/backend/uploads/data.xlsx
@@ -1,62 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29130"/>
-  <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andrescortesdev/Riwi/celsia/v2/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{AE0C68B0-73E6-BA48-845F-50FC557F2199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D6E18937-A1A0-4F2F-838B-66B2816A8F24}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="623">
-  <si>
-    <t>ID de la Transacción</t>
-  </si>
-  <si>
-    <t>Fecha y Hora de la Transacción</t>
-  </si>
-  <si>
-    <t>Monto de la Transacción</t>
-  </si>
-  <si>
-    <t>Estado de la Transacción</t>
-  </si>
-  <si>
-    <t>Tipo de Transacción</t>
-  </si>
-  <si>
-    <t>Nombre del Cliente</t>
-  </si>
-  <si>
-    <t>Número de Identificación</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="623">
+  <si>
+    <t xml:space="preserve">ID de la Transacción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fecha y Hora de la Transacción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monto de la Transacción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estado de la Transacción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de Transacción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nombre del Cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Número de Identificación</t>
   </si>
   <si>
     <t>Dirección</t>
@@ -65,22 +45,22 @@
     <t>Teléfono</t>
   </si>
   <si>
-    <t>Correo Electrónico</t>
-  </si>
-  <si>
-    <t>Plataforma Utilizada</t>
-  </si>
-  <si>
-    <t>Número de Factura</t>
-  </si>
-  <si>
-    <t>Periodo de Facturación</t>
-  </si>
-  <si>
-    <t>Monto Facturado</t>
-  </si>
-  <si>
-    <t>Monto Pagado</t>
+    <t xml:space="preserve">Correo Electrónico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plataforma Utilizada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Número de Factura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Periodo de Facturación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monto Facturado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monto Pagado</t>
   </si>
   <si>
     <t>TXN001</t>
@@ -89,13 +69,13 @@
     <t>Pendiente</t>
   </si>
   <si>
-    <t>Pago de Factura</t>
-  </si>
-  <si>
-    <t>Angel Daniel</t>
-  </si>
-  <si>
-    <t>USNS Davis
+    <t xml:space="preserve">Pago de Factura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angel Daniel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USNS Davis
 FPO AP 78518</t>
   </si>
   <si>
@@ -117,10 +97,10 @@
     <t>TXN002</t>
   </si>
   <si>
-    <t>Matthew Wilson</t>
-  </si>
-  <si>
-    <t>42023 Barrett Path Suite 281
+    <t xml:space="preserve">Matthew Wilson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42023 Barrett Path Suite 281
 Jeremyborough, OH 72889</t>
   </si>
   <si>
@@ -142,10 +122,10 @@
     <t>Fallida</t>
   </si>
   <si>
-    <t>Jennifer Phelps</t>
-  </si>
-  <si>
-    <t>392 Smith Corners Apt. 737
+    <t xml:space="preserve">Jennifer Phelps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">392 Smith Corners Apt. 737
 East Angeltown, MO 64086</t>
   </si>
   <si>
@@ -161,10 +141,10 @@
     <t>TXN004</t>
   </si>
   <si>
-    <t>Jonathan Cook</t>
-  </si>
-  <si>
-    <t>657 Landry Way Suite 966
+    <t xml:space="preserve">Jonathan Cook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">657 Landry Way Suite 966
 Robinsonfurt, CA 22461</t>
   </si>
   <si>
@@ -186,10 +166,10 @@
     <t>Completada</t>
   </si>
   <si>
-    <t>Lindsay Garcia</t>
-  </si>
-  <si>
-    <t>906 Justin Locks Apt. 838
+    <t xml:space="preserve">Lindsay Garcia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">906 Justin Locks Apt. 838
 Port Timothyview, AR 68865</t>
   </si>
   <si>
@@ -205,10 +185,10 @@
     <t>TXN006</t>
   </si>
   <si>
-    <t>Eric Klein</t>
-  </si>
-  <si>
-    <t>0571 Carroll Cliffs
+    <t xml:space="preserve">Eric Klein</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0571 Carroll Cliffs
 Davisstad, WI 00721</t>
   </si>
   <si>
@@ -224,10 +204,10 @@
     <t>TXN007</t>
   </si>
   <si>
-    <t>Ashley Adams</t>
-  </si>
-  <si>
-    <t>660 Marcus Camp Suite 262
+    <t xml:space="preserve">Ashley Adams</t>
+  </si>
+  <si>
+    <t xml:space="preserve">660 Marcus Camp Suite 262
 Port Stevenmouth, NC 10819</t>
   </si>
   <si>
@@ -243,10 +223,10 @@
     <t>TXN008</t>
   </si>
   <si>
-    <t>Meghan Nguyen</t>
-  </si>
-  <si>
-    <t>259 Jared Manor
+    <t xml:space="preserve">Meghan Nguyen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">259 Jared Manor
 Brownville, AZ 52844</t>
   </si>
   <si>
@@ -262,10 +242,10 @@
     <t>TXN009</t>
   </si>
   <si>
-    <t>Ryan Richards</t>
-  </si>
-  <si>
-    <t>695 Francis Cliffs
+    <t xml:space="preserve">Ryan Richards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">695 Francis Cliffs
 Port Bryantown, VT 33873</t>
   </si>
   <si>
@@ -281,10 +261,10 @@
     <t>TXN010</t>
   </si>
   <si>
-    <t>Janice Alexander</t>
-  </si>
-  <si>
-    <t>81268 Hamilton Fort
+    <t xml:space="preserve">Janice Alexander</t>
+  </si>
+  <si>
+    <t xml:space="preserve">81268 Hamilton Fort
 Fitzgeraldfort, ID 71489</t>
   </si>
   <si>
@@ -300,10 +280,10 @@
     <t>TXN011</t>
   </si>
   <si>
-    <t>Katherine Dunn</t>
-  </si>
-  <si>
-    <t>837 Schneider Spur Suite 656
+    <t xml:space="preserve">Katherine Dunn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">837 Schneider Spur Suite 656
 Darrellmouth, WI 33323</t>
   </si>
   <si>
@@ -319,10 +299,10 @@
     <t>TXN012</t>
   </si>
   <si>
-    <t>Brett Odom</t>
-  </si>
-  <si>
-    <t>952 Barbara Turnpike
+    <t xml:space="preserve">Brett Odom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">952 Barbara Turnpike
 Jacquelinebury, MO 71346</t>
   </si>
   <si>
@@ -338,10 +318,10 @@
     <t>TXN013</t>
   </si>
   <si>
-    <t>Jenna Scott</t>
-  </si>
-  <si>
-    <t>Unit 1694 Box 1865
+    <t xml:space="preserve">Jenna Scott</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit 1694 Box 1865
 DPO AE 26667</t>
   </si>
   <si>
@@ -357,10 +337,10 @@
     <t>TXN014</t>
   </si>
   <si>
-    <t>Andrew Johns</t>
-  </si>
-  <si>
-    <t>62457 Booth Mews Apt. 453
+    <t xml:space="preserve">Andrew Johns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">62457 Booth Mews Apt. 453
 Lake Vincentport, DE 49208</t>
   </si>
   <si>
@@ -376,10 +356,10 @@
     <t>TXN015</t>
   </si>
   <si>
-    <t>Christine Curtis</t>
-  </si>
-  <si>
-    <t>2480 Jesse Unions Suite 534
+    <t xml:space="preserve">Christine Curtis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2480 Jesse Unions Suite 534
 East Antonioshire, MS 71510</t>
   </si>
   <si>
@@ -395,10 +375,10 @@
     <t>TXN016</t>
   </si>
   <si>
-    <t>Madison Jones</t>
-  </si>
-  <si>
-    <t>USNS Ferguson
+    <t xml:space="preserve">Madison Jones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USNS Ferguson
 FPO AP 50263</t>
   </si>
   <si>
@@ -414,10 +394,10 @@
     <t>TXN017</t>
   </si>
   <si>
-    <t>Tracy Simmons</t>
-  </si>
-  <si>
-    <t>76775 Jennifer Orchard Apt. 758
+    <t xml:space="preserve">Tracy Simmons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">76775 Jennifer Orchard Apt. 758
 Port Lance, NH 53890</t>
   </si>
   <si>
@@ -433,10 +413,10 @@
     <t>TXN018</t>
   </si>
   <si>
-    <t>Shelby Wolf</t>
-  </si>
-  <si>
-    <t>613 Billy Radial Suite 171
+    <t xml:space="preserve">Shelby Wolf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">613 Billy Radial Suite 171
 South Benjamin, WY 15230</t>
   </si>
   <si>
@@ -452,10 +432,10 @@
     <t>TXN019</t>
   </si>
   <si>
-    <t>Kyle Jackson</t>
-  </si>
-  <si>
-    <t>24896 Helen Rapid Suite 758
+    <t xml:space="preserve">Kyle Jackson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24896 Helen Rapid Suite 758
 New Joseph, MN 97017</t>
   </si>
   <si>
@@ -471,10 +451,10 @@
     <t>TXN020</t>
   </si>
   <si>
-    <t>Linda Shepard</t>
-  </si>
-  <si>
-    <t>4947 Reynolds Islands
+    <t xml:space="preserve">Linda Shepard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4947 Reynolds Islands
 Kathleenburgh, DE 96988</t>
   </si>
   <si>
@@ -490,10 +470,10 @@
     <t>TXN021</t>
   </si>
   <si>
-    <t>Kathleen Brady</t>
-  </si>
-  <si>
-    <t>Unit 6453 Box 5308
+    <t xml:space="preserve">Kathleen Brady</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit 6453 Box 5308
 DPO AA 48049</t>
   </si>
   <si>
@@ -509,10 +489,10 @@
     <t>TXN022</t>
   </si>
   <si>
-    <t>Bobby Luna</t>
-  </si>
-  <si>
-    <t>2923 Michael Fords Suite 316
+    <t xml:space="preserve">Bobby Luna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2923 Michael Fords Suite 316
 Dustinton, IN 31032</t>
   </si>
   <si>
@@ -528,10 +508,10 @@
     <t>TXN023</t>
   </si>
   <si>
-    <t>Richard Lopez</t>
-  </si>
-  <si>
-    <t>6875 Hill Forks
+    <t xml:space="preserve">Richard Lopez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6875 Hill Forks
 Teresaland, AL 58910</t>
   </si>
   <si>
@@ -547,10 +527,10 @@
     <t>TXN024</t>
   </si>
   <si>
-    <t>Ralph Bush</t>
-  </si>
-  <si>
-    <t>03975 Mills Square Apt. 322
+    <t xml:space="preserve">Ralph Bush</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03975 Mills Square Apt. 322
 Port Claudia, MI 34792</t>
   </si>
   <si>
@@ -566,10 +546,10 @@
     <t>TXN025</t>
   </si>
   <si>
-    <t>David Webb</t>
-  </si>
-  <si>
-    <t>3613 Laura Ridges Suite 762
+    <t xml:space="preserve">David Webb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3613 Laura Ridges Suite 762
 South Theresa, VA 98493</t>
   </si>
   <si>
@@ -585,10 +565,10 @@
     <t>TXN026</t>
   </si>
   <si>
-    <t>Kim Russell</t>
-  </si>
-  <si>
-    <t>887 Kelley Walk Apt. 960
+    <t xml:space="preserve">Kim Russell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">887 Kelley Walk Apt. 960
 East Martha, CT 59649</t>
   </si>
   <si>
@@ -604,10 +584,10 @@
     <t>TXN027</t>
   </si>
   <si>
-    <t>Michael Holt</t>
-  </si>
-  <si>
-    <t>3499 David Lake Suite 745
+    <t xml:space="preserve">Michael Holt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3499 David Lake Suite 745
 South Dylan, AK 03041</t>
   </si>
   <si>
@@ -623,10 +603,10 @@
     <t>TXN028</t>
   </si>
   <si>
-    <t>Mr. Justin Cook</t>
-  </si>
-  <si>
-    <t>Unit 9907 Box 4757
+    <t xml:space="preserve">Mr. Justin Cook</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit 9907 Box 4757
 DPO AE 46640</t>
   </si>
   <si>
@@ -642,10 +622,10 @@
     <t>TXN029</t>
   </si>
   <si>
-    <t>Timothy Wood</t>
-  </si>
-  <si>
-    <t>836 Bates Points
+    <t xml:space="preserve">Timothy Wood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">836 Bates Points
 Port Andrewshire, GA 83721</t>
   </si>
   <si>
@@ -661,10 +641,10 @@
     <t>TXN030</t>
   </si>
   <si>
-    <t>Yolanda Hines</t>
-  </si>
-  <si>
-    <t>812 Mccarthy Viaduct Apt. 376
+    <t xml:space="preserve">Yolanda Hines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">812 Mccarthy Viaduct Apt. 376
 Kristinamouth, AL 43563</t>
   </si>
   <si>
@@ -680,10 +660,10 @@
     <t>TXN031</t>
   </si>
   <si>
-    <t>Jasmine Kelly</t>
-  </si>
-  <si>
-    <t>697 Reynolds Dam Apt. 423
+    <t xml:space="preserve">Jasmine Kelly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">697 Reynolds Dam Apt. 423
 Jacobland, MO 89387</t>
   </si>
   <si>
@@ -699,10 +679,10 @@
     <t>TXN032</t>
   </si>
   <si>
-    <t>Robert Smith</t>
-  </si>
-  <si>
-    <t>Unit 2774 Box 4368
+    <t xml:space="preserve">Robert Smith</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit 2774 Box 4368
 DPO AE 01041</t>
   </si>
   <si>
@@ -718,10 +698,10 @@
     <t>TXN033</t>
   </si>
   <si>
-    <t>Jonathan Smith</t>
-  </si>
-  <si>
-    <t>322 Smith Pines Suite 052
+    <t xml:space="preserve">Jonathan Smith</t>
+  </si>
+  <si>
+    <t xml:space="preserve">322 Smith Pines Suite 052
 Lake Scotthaven, NM 11543</t>
   </si>
   <si>
@@ -737,10 +717,10 @@
     <t>TXN034</t>
   </si>
   <si>
-    <t>Erin Marshall</t>
-  </si>
-  <si>
-    <t>04382 Edward Mountains Suite 369
+    <t xml:space="preserve">Erin Marshall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04382 Edward Mountains Suite 369
 Georgeberg, ME 94518</t>
   </si>
   <si>
@@ -756,10 +736,10 @@
     <t>TXN035</t>
   </si>
   <si>
-    <t>Mark Ford</t>
-  </si>
-  <si>
-    <t>07900 Friedman Ferry Suite 170
+    <t xml:space="preserve">Mark Ford</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07900 Friedman Ferry Suite 170
 South Christina, WV 53142</t>
   </si>
   <si>
@@ -775,10 +755,10 @@
     <t>TXN036</t>
   </si>
   <si>
-    <t>Cynthia Lee</t>
-  </si>
-  <si>
-    <t>368 Jones Estates Apt. 059
+    <t xml:space="preserve">Cynthia Lee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">368 Jones Estates Apt. 059
 Jonesstad, NY 59968</t>
   </si>
   <si>
@@ -794,10 +774,10 @@
     <t>TXN037</t>
   </si>
   <si>
-    <t>Sean Hood</t>
-  </si>
-  <si>
-    <t>7426 Middleton Hill Suite 303
+    <t xml:space="preserve">Sean Hood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7426 Middleton Hill Suite 303
 Millerview, CO 23232</t>
   </si>
   <si>
@@ -813,10 +793,10 @@
     <t>TXN038</t>
   </si>
   <si>
-    <t>Kim Stephens</t>
-  </si>
-  <si>
-    <t>12967 Ryan Shoals Apt. 994
+    <t xml:space="preserve">Kim Stephens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12967 Ryan Shoals Apt. 994
 Port Jesse, MO 86007</t>
   </si>
   <si>
@@ -832,10 +812,10 @@
     <t>TXN039</t>
   </si>
   <si>
-    <t>Adam Mckinney</t>
-  </si>
-  <si>
-    <t>572 Tammy Forest
+    <t xml:space="preserve">Adam Mckinney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">572 Tammy Forest
 Youngside, SD 92567</t>
   </si>
   <si>
@@ -851,10 +831,10 @@
     <t>TXN040</t>
   </si>
   <si>
-    <t>Valerie Brown</t>
-  </si>
-  <si>
-    <t>2739 Hood Rest Apt. 962
+    <t xml:space="preserve">Valerie Brown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2739 Hood Rest Apt. 962
 Johnburgh, UT 27169</t>
   </si>
   <si>
@@ -870,10 +850,10 @@
     <t>TXN041</t>
   </si>
   <si>
-    <t>Jason Pace</t>
-  </si>
-  <si>
-    <t>19964 Edwards Pines
+    <t xml:space="preserve">Jason Pace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19964 Edwards Pines
 South Jeremystad, AZ 79080</t>
   </si>
   <si>
@@ -889,10 +869,10 @@
     <t>TXN042</t>
   </si>
   <si>
-    <t>Gregory Anderson</t>
-  </si>
-  <si>
-    <t>5395 Brandon Freeway Apt. 858
+    <t xml:space="preserve">Gregory Anderson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5395 Brandon Freeway Apt. 858
 North Melissa, OR 60184</t>
   </si>
   <si>
@@ -908,10 +888,10 @@
     <t>TXN043</t>
   </si>
   <si>
-    <t>Rebecca Avila</t>
-  </si>
-  <si>
-    <t>78969 Mcguire Springs Suite 562
+    <t xml:space="preserve">Rebecca Avila</t>
+  </si>
+  <si>
+    <t xml:space="preserve">78969 Mcguire Springs Suite 562
 Port Christopher, NJ 29478</t>
   </si>
   <si>
@@ -927,10 +907,10 @@
     <t>TXN044</t>
   </si>
   <si>
-    <t>Morgan Leon</t>
-  </si>
-  <si>
-    <t>853 Virginia Cape Suite 757
+    <t xml:space="preserve">Morgan Leon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">853 Virginia Cape Suite 757
 Wilsonport, SC 89614</t>
   </si>
   <si>
@@ -946,10 +926,10 @@
     <t>TXN045</t>
   </si>
   <si>
-    <t>Fernando Hunt</t>
-  </si>
-  <si>
-    <t>9609 Conner Track Apt. 859
+    <t xml:space="preserve">Fernando Hunt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9609 Conner Track Apt. 859
 Kristenberg, MD 40765</t>
   </si>
   <si>
@@ -965,10 +945,10 @@
     <t>TXN046</t>
   </si>
   <si>
-    <t>Jason Luna</t>
-  </si>
-  <si>
-    <t>204 Laura Hill
+    <t xml:space="preserve">Jason Luna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">204 Laura Hill
 Craigland, OK 08760</t>
   </si>
   <si>
@@ -984,10 +964,10 @@
     <t>TXN047</t>
   </si>
   <si>
-    <t>Gregory Howell</t>
-  </si>
-  <si>
-    <t>036 Tyler Groves Suite 302
+    <t xml:space="preserve">Gregory Howell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">036 Tyler Groves Suite 302
 Danielsfurt, WV 45483</t>
   </si>
   <si>
@@ -1003,10 +983,10 @@
     <t>TXN048</t>
   </si>
   <si>
-    <t>Miguel Sharp MD</t>
-  </si>
-  <si>
-    <t>47921 Johnson Expressway Suite 742
+    <t xml:space="preserve">Miguel Sharp MD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47921 Johnson Expressway Suite 742
 Oliviaport, PA 16931</t>
   </si>
   <si>
@@ -1022,10 +1002,10 @@
     <t>TXN049</t>
   </si>
   <si>
-    <t>Stephanie Acosta</t>
-  </si>
-  <si>
-    <t>7067 Henderson Knoll
+    <t xml:space="preserve">Stephanie Acosta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7067 Henderson Knoll
 Joshuashire, NJ 84213</t>
   </si>
   <si>
@@ -1041,10 +1021,10 @@
     <t>TXN050</t>
   </si>
   <si>
-    <t>Julia Davis</t>
-  </si>
-  <si>
-    <t>0246 Brown Roads Suite 606
+    <t xml:space="preserve">Julia Davis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0246 Brown Roads Suite 606
 North Luisburgh, WI 38462</t>
   </si>
   <si>
@@ -1060,10 +1040,10 @@
     <t>TXN051</t>
   </si>
   <si>
-    <t>Amy Woods</t>
-  </si>
-  <si>
-    <t>247 Sheila Centers
+    <t xml:space="preserve">Amy Woods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">247 Sheila Centers
 North Troybury, WA 43836</t>
   </si>
   <si>
@@ -1079,10 +1059,10 @@
     <t>TXN052</t>
   </si>
   <si>
-    <t>Julie Dunn</t>
-  </si>
-  <si>
-    <t>758 Ruth Mall
+    <t xml:space="preserve">Julie Dunn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">758 Ruth Mall
 Briggstown, MA 48538</t>
   </si>
   <si>
@@ -1098,10 +1078,10 @@
     <t>TXN053</t>
   </si>
   <si>
-    <t>Nicole Mcdonald</t>
-  </si>
-  <si>
-    <t>7229 Michelle Forges Suite 411
+    <t xml:space="preserve">Nicole Mcdonald</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7229 Michelle Forges Suite 411
 Hardyview, VT 06858</t>
   </si>
   <si>
@@ -1117,10 +1097,10 @@
     <t>TXN054</t>
   </si>
   <si>
-    <t>Jennifer Mendoza</t>
-  </si>
-  <si>
-    <t>11916 Katherine Creek
+    <t xml:space="preserve">Jennifer Mendoza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11916 Katherine Creek
 Kathleenport, ND 68479</t>
   </si>
   <si>
@@ -1136,10 +1116,10 @@
     <t>TXN055</t>
   </si>
   <si>
-    <t>Rachel Fisher</t>
-  </si>
-  <si>
-    <t>38507 Newman Loop Suite 268
+    <t xml:space="preserve">Rachel Fisher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38507 Newman Loop Suite 268
 Tommyberg, UT 25108</t>
   </si>
   <si>
@@ -1155,10 +1135,10 @@
     <t>TXN056</t>
   </si>
   <si>
-    <t>Jorge Thomas</t>
-  </si>
-  <si>
-    <t>013 Tabitha Cliff
+    <t xml:space="preserve">Jorge Thomas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">013 Tabitha Cliff
 Stevenmouth, NJ 04089</t>
   </si>
   <si>
@@ -1174,10 +1154,10 @@
     <t>TXN057</t>
   </si>
   <si>
-    <t>Robert Hicks</t>
-  </si>
-  <si>
-    <t>1639 Delacruz Park
+    <t xml:space="preserve">Robert Hicks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1639 Delacruz Park
 East Linda, DC 18242</t>
   </si>
   <si>
@@ -1193,10 +1173,10 @@
     <t>TXN058</t>
   </si>
   <si>
-    <t>Terry Watson</t>
-  </si>
-  <si>
-    <t>0047 Lori Square
+    <t xml:space="preserve">Terry Watson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0047 Lori Square
 East Josechester, KS 29146</t>
   </si>
   <si>
@@ -1212,10 +1192,10 @@
     <t>TXN059</t>
   </si>
   <si>
-    <t>Carlos Wood</t>
-  </si>
-  <si>
-    <t>53828 Laura Spurs
+    <t xml:space="preserve">Carlos Wood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">53828 Laura Spurs
 Lauraville, DE 53316</t>
   </si>
   <si>
@@ -1231,10 +1211,10 @@
     <t>TXN060</t>
   </si>
   <si>
-    <t>Richard Weiss</t>
-  </si>
-  <si>
-    <t>316 Robert Dam
+    <t xml:space="preserve">Richard Weiss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">316 Robert Dam
 North Christina, MA 15552</t>
   </si>
   <si>
@@ -1250,10 +1230,10 @@
     <t>TXN061</t>
   </si>
   <si>
-    <t>Sarah Clark</t>
-  </si>
-  <si>
-    <t>04967 Nguyen Circle Suite 871
+    <t xml:space="preserve">Sarah Clark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04967 Nguyen Circle Suite 871
 Lake Andrea, NY 87021</t>
   </si>
   <si>
@@ -1269,10 +1249,10 @@
     <t>TXN062</t>
   </si>
   <si>
-    <t>Briana Wu</t>
-  </si>
-  <si>
-    <t>534 Campbell View
+    <t xml:space="preserve">Briana Wu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">534 Campbell View
 Sandersland, FL 59798</t>
   </si>
   <si>
@@ -1288,10 +1268,10 @@
     <t>TXN063</t>
   </si>
   <si>
-    <t>Raven Jordan</t>
-  </si>
-  <si>
-    <t>6132 Spencer Corner Apt. 383
+    <t xml:space="preserve">Raven Jordan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6132 Spencer Corner Apt. 383
 Lake Loriberg, MA 96874</t>
   </si>
   <si>
@@ -1307,10 +1287,10 @@
     <t>TXN064</t>
   </si>
   <si>
-    <t>Angelica Gibbs</t>
-  </si>
-  <si>
-    <t>68574 Coleman Villages Suite 522
+    <t xml:space="preserve">Angelica Gibbs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">68574 Coleman Villages Suite 522
 North Erikaton, CA 83413</t>
   </si>
   <si>
@@ -1326,10 +1306,10 @@
     <t>TXN065</t>
   </si>
   <si>
-    <t>Tammy Jacobs</t>
-  </si>
-  <si>
-    <t>57458 Collier Junctions Suite 288
+    <t xml:space="preserve">Tammy Jacobs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">57458 Collier Junctions Suite 288
 Lake Nicholas, CT 00530</t>
   </si>
   <si>
@@ -1345,10 +1325,10 @@
     <t>TXN066</t>
   </si>
   <si>
-    <t>Michael Evans</t>
-  </si>
-  <si>
-    <t>921 Ramirez Mount
+    <t xml:space="preserve">Michael Evans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">921 Ramirez Mount
 New Anthonyville, ND 52047</t>
   </si>
   <si>
@@ -1364,10 +1344,10 @@
     <t>TXN067</t>
   </si>
   <si>
-    <t>Tony Pham</t>
-  </si>
-  <si>
-    <t>Unit 3715 Box 5620
+    <t xml:space="preserve">Tony Pham</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit 3715 Box 5620
 DPO AA 18266</t>
   </si>
   <si>
@@ -1383,10 +1363,10 @@
     <t>TXN068</t>
   </si>
   <si>
-    <t>Miss Carrie Underwood</t>
-  </si>
-  <si>
-    <t>USNV Morris
+    <t xml:space="preserve">Miss Carrie Underwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USNV Morris
 FPO AA 49085</t>
   </si>
   <si>
@@ -1402,10 +1382,10 @@
     <t>TXN069</t>
   </si>
   <si>
-    <t>Ryan Russell</t>
-  </si>
-  <si>
-    <t>70003 Tiffany Drives
+    <t xml:space="preserve">Ryan Russell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70003 Tiffany Drives
 Robertchester, IA 05998</t>
   </si>
   <si>
@@ -1421,10 +1401,10 @@
     <t>TXN070</t>
   </si>
   <si>
-    <t>Kimberly Bennett</t>
-  </si>
-  <si>
-    <t>70851 Daniel Station Apt. 975
+    <t xml:space="preserve">Kimberly Bennett</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70851 Daniel Station Apt. 975
 Hernandezton, IL 77476</t>
   </si>
   <si>
@@ -1440,10 +1420,10 @@
     <t>TXN071</t>
   </si>
   <si>
-    <t>Joshua Neal</t>
-  </si>
-  <si>
-    <t>1324 William Glens
+    <t xml:space="preserve">Joshua Neal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1324 William Glens
 New Jenniferland, IL 16679</t>
   </si>
   <si>
@@ -1459,10 +1439,10 @@
     <t>TXN072</t>
   </si>
   <si>
-    <t>Robert Rodriguez</t>
-  </si>
-  <si>
-    <t>9483 Patricia Greens Suite 612
+    <t xml:space="preserve">Robert Rodriguez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9483 Patricia Greens Suite 612
 West Daniel, CT 37484</t>
   </si>
   <si>
@@ -1478,10 +1458,10 @@
     <t>TXN073</t>
   </si>
   <si>
-    <t>Blake Ford</t>
-  </si>
-  <si>
-    <t>933 Casey Court Apt. 193
+    <t xml:space="preserve">Blake Ford</t>
+  </si>
+  <si>
+    <t xml:space="preserve">933 Casey Court Apt. 193
 Lake Douglas, AL 33325</t>
   </si>
   <si>
@@ -1497,10 +1477,10 @@
     <t>TXN074</t>
   </si>
   <si>
-    <t>Chad Garcia</t>
-  </si>
-  <si>
-    <t>195 Rollins Land Suite 478
+    <t xml:space="preserve">Chad Garcia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">195 Rollins Land Suite 478
 North Angelastad, IN 84674</t>
   </si>
   <si>
@@ -1516,10 +1496,10 @@
     <t>TXN075</t>
   </si>
   <si>
-    <t>Autumn Webb</t>
-  </si>
-  <si>
-    <t>198 Frazier Branch Suite 399
+    <t xml:space="preserve">Autumn Webb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">198 Frazier Branch Suite 399
 South Sharon, AR 75490</t>
   </si>
   <si>
@@ -1535,10 +1515,10 @@
     <t>TXN076</t>
   </si>
   <si>
-    <t>Elizabeth Singleton</t>
-  </si>
-  <si>
-    <t>87020 Horton Valleys
+    <t xml:space="preserve">Elizabeth Singleton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">87020 Horton Valleys
 Rodriguezfurt, WV 03348</t>
   </si>
   <si>
@@ -1554,10 +1534,10 @@
     <t>TXN077</t>
   </si>
   <si>
-    <t>Sarah Thompson</t>
-  </si>
-  <si>
-    <t>Unit 0218 Box 2805
+    <t xml:space="preserve">Sarah Thompson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit 0218 Box 2805
 DPO AA 08015</t>
   </si>
   <si>
@@ -1573,10 +1553,10 @@
     <t>TXN078</t>
   </si>
   <si>
-    <t>Sarah Martin</t>
-  </si>
-  <si>
-    <t>5963 Strong Points
+    <t xml:space="preserve">Sarah Martin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5963 Strong Points
 Lake Kayla, SC 51830</t>
   </si>
   <si>
@@ -1592,10 +1572,10 @@
     <t>TXN079</t>
   </si>
   <si>
-    <t>Pamela Herrera</t>
-  </si>
-  <si>
-    <t>3416 Gregory Rapids Suite 629
+    <t xml:space="preserve">Pamela Herrera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3416 Gregory Rapids Suite 629
 North Nicolehaven, IL 93329</t>
   </si>
   <si>
@@ -1611,10 +1591,10 @@
     <t>TXN080</t>
   </si>
   <si>
-    <t>Shannon Horn</t>
-  </si>
-  <si>
-    <t>USNS Buchanan
+    <t xml:space="preserve">Shannon Horn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USNS Buchanan
 FPO AA 82885</t>
   </si>
   <si>
@@ -1630,10 +1610,10 @@
     <t>TXN081</t>
   </si>
   <si>
-    <t>Christopher Edwards</t>
-  </si>
-  <si>
-    <t>32230 Jeffery Via Apt. 616
+    <t xml:space="preserve">Christopher Edwards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32230 Jeffery Via Apt. 616
 West Tanya, WA 77567</t>
   </si>
   <si>
@@ -1649,10 +1629,10 @@
     <t>TXN082</t>
   </si>
   <si>
-    <t>Brandon Hester</t>
-  </si>
-  <si>
-    <t>0169 Summers Vista
+    <t xml:space="preserve">Brandon Hester</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0169 Summers Vista
 West Stuart, UT 98685</t>
   </si>
   <si>
@@ -1668,10 +1648,10 @@
     <t>TXN083</t>
   </si>
   <si>
-    <t>Mariah Jackson</t>
-  </si>
-  <si>
-    <t>558 Bryan Isle
+    <t xml:space="preserve">Mariah Jackson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">558 Bryan Isle
 New Raymond, AL 55316</t>
   </si>
   <si>
@@ -1687,10 +1667,10 @@
     <t>TXN084</t>
   </si>
   <si>
-    <t>Carol Lawson</t>
-  </si>
-  <si>
-    <t>747 Miller Point
+    <t xml:space="preserve">Carol Lawson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">747 Miller Point
 Georgeton, UT 90920</t>
   </si>
   <si>
@@ -1706,10 +1686,10 @@
     <t>TXN085</t>
   </si>
   <si>
-    <t>Heather Collins</t>
-  </si>
-  <si>
-    <t>7878 Nelson Stravenue
+    <t xml:space="preserve">Heather Collins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7878 Nelson Stravenue
 New Jacob, NE 62801</t>
   </si>
   <si>
@@ -1725,10 +1705,10 @@
     <t>TXN086</t>
   </si>
   <si>
-    <t>Joshua Delgado</t>
-  </si>
-  <si>
-    <t>741 Morgan Underpass
+    <t xml:space="preserve">Joshua Delgado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">741 Morgan Underpass
 South Sheila, IL 16740</t>
   </si>
   <si>
@@ -1744,10 +1724,10 @@
     <t>TXN087</t>
   </si>
   <si>
-    <t>Jerry Greene</t>
-  </si>
-  <si>
-    <t>60823 Lauren Wall Apt. 074
+    <t xml:space="preserve">Jerry Greene</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60823 Lauren Wall Apt. 074
 New Kellyside, MI 21097</t>
   </si>
   <si>
@@ -1763,10 +1743,10 @@
     <t>TXN088</t>
   </si>
   <si>
-    <t>Connor Wagner</t>
-  </si>
-  <si>
-    <t>506 Brandy Rapid
+    <t xml:space="preserve">Connor Wagner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">506 Brandy Rapid
 Dawsonberg, RI 42470</t>
   </si>
   <si>
@@ -1782,10 +1762,10 @@
     <t>TXN089</t>
   </si>
   <si>
-    <t>Marcia Randolph</t>
-  </si>
-  <si>
-    <t>327 Roberts Neck
+    <t xml:space="preserve">Marcia Randolph</t>
+  </si>
+  <si>
+    <t xml:space="preserve">327 Roberts Neck
 Gonzalezshire, WA 18952</t>
   </si>
   <si>
@@ -1801,10 +1781,10 @@
     <t>TXN090</t>
   </si>
   <si>
-    <t>John Price</t>
-  </si>
-  <si>
-    <t>PSC 5622, Box 3709
+    <t xml:space="preserve">John Price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PSC 5622, Box 3709
 APO AA 38900</t>
   </si>
   <si>
@@ -1820,10 +1800,10 @@
     <t>TXN091</t>
   </si>
   <si>
-    <t>Bill Hopkins</t>
-  </si>
-  <si>
-    <t>54675 Matthew Key
+    <t xml:space="preserve">Bill Hopkins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">54675 Matthew Key
 Torresstad, ME 64087</t>
   </si>
   <si>
@@ -1839,10 +1819,10 @@
     <t>TXN092</t>
   </si>
   <si>
-    <t>Ryan Harrison</t>
-  </si>
-  <si>
-    <t>66252 Trevor Harbor Apt. 887
+    <t xml:space="preserve">Ryan Harrison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">66252 Trevor Harbor Apt. 887
 Lake Ambertown, TN 81820</t>
   </si>
   <si>
@@ -1858,10 +1838,10 @@
     <t>TXN093</t>
   </si>
   <si>
-    <t>Donald Young</t>
-  </si>
-  <si>
-    <t>223 Dawson Mall Suite 571
+    <t xml:space="preserve">Donald Young</t>
+  </si>
+  <si>
+    <t xml:space="preserve">223 Dawson Mall Suite 571
 Smithburgh, MS 75952</t>
   </si>
   <si>
@@ -1877,10 +1857,10 @@
     <t>TXN094</t>
   </si>
   <si>
-    <t>Louis Gilbert</t>
-  </si>
-  <si>
-    <t>530 Brown Corner
+    <t xml:space="preserve">Louis Gilbert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">530 Brown Corner
 Thompsontown, WV 70738</t>
   </si>
   <si>
@@ -1896,10 +1876,10 @@
     <t>TXN095</t>
   </si>
   <si>
-    <t>Marcus Martin</t>
-  </si>
-  <si>
-    <t>PSC 6227, Box 1600
+    <t xml:space="preserve">Marcus Martin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PSC 6227, Box 1600
 APO AP 14578</t>
   </si>
   <si>
@@ -1915,10 +1895,10 @@
     <t>TXN096</t>
   </si>
   <si>
-    <t>Sharon Ingram</t>
-  </si>
-  <si>
-    <t>132 Vargas Turnpike
+    <t xml:space="preserve">Sharon Ingram</t>
+  </si>
+  <si>
+    <t xml:space="preserve">132 Vargas Turnpike
 Danielbury, DE 40715</t>
   </si>
   <si>
@@ -1934,10 +1914,10 @@
     <t>TXN097</t>
   </si>
   <si>
-    <t>Kyle Martinez</t>
-  </si>
-  <si>
-    <t>USS Greene
+    <t xml:space="preserve">Kyle Martinez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USS Greene
 FPO AA 26511</t>
   </si>
   <si>
@@ -1953,10 +1933,10 @@
     <t>TXN098</t>
   </si>
   <si>
-    <t>Elizabeth Rodriguez</t>
-  </si>
-  <si>
-    <t>3551 Rodriguez Port Apt. 808
+    <t xml:space="preserve">Elizabeth Rodriguez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3551 Rodriguez Port Apt. 808
 Lake Charles, WI 24322</t>
   </si>
   <si>
@@ -1972,10 +1952,10 @@
     <t>TXN099</t>
   </si>
   <si>
-    <t>Christopher Gomez</t>
-  </si>
-  <si>
-    <t>875 Jennifer Oval Suite 067
+    <t xml:space="preserve">Christopher Gomez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">875 Jennifer Oval Suite 067
 West Phillipmouth, IL 91337</t>
   </si>
   <si>
@@ -1991,10 +1971,10 @@
     <t>TXN100</t>
   </si>
   <si>
-    <t>Brian Morton</t>
-  </si>
-  <si>
-    <t>431 Rodriguez Estate Suite 894
+    <t xml:space="preserve">Brian Morton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">431 Rodriguez Estate Suite 894
 New Christopherview, TN 74616</t>
   </si>
   <si>
@@ -2010,25 +1990,29 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11.000000"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2041,28 +2025,29 @@
   </fills>
   <borders count="1">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="4">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2074,10 +2059,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2115,18 +2100,18 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Angsana New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -2149,19 +2134,18 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Thai" typeface="Cordia New"/>
         <a:font script="Ethi" typeface="Nyala"/>
         <a:font script="Beng" typeface="Vrinda"/>
         <a:font script="Gujr" typeface="Shruti"/>
@@ -2184,10 +2168,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2359,31 +2342,250 @@
 </a:theme>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme 2007 - 2010">
+  <a:themeElements>
+    <a:clrScheme name="Office 2007 - 2010">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office 2007 - 2010">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office 2007 - 2010">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q101"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="57.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="42.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="22" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="52" bestFit="1" customWidth="1"/>
+    <col bestFit="1" customWidth="1" min="1" max="1" width="19"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" width="28.7109375"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" width="23.28515625"/>
+    <col bestFit="1" customWidth="1" min="4" max="4" width="23.140625"/>
+    <col bestFit="1" customWidth="1" min="5" max="5" width="18.85546875"/>
+    <col bestFit="1" customWidth="1" min="6" max="6" width="22.140625"/>
+    <col bestFit="1" customWidth="1" min="7" max="7" width="24.140625"/>
+    <col bestFit="1" customWidth="1" min="8" max="8" width="57.42578125"/>
+    <col bestFit="1" customWidth="1" min="9" max="9" width="24"/>
+    <col bestFit="1" customWidth="1" min="10" max="10" width="42.42578125"/>
+    <col bestFit="1" customWidth="1" min="11" max="11" width="19.7109375"/>
+    <col bestFit="1" customWidth="1" min="12" max="12" width="18.42578125"/>
+    <col bestFit="1" customWidth="1" min="13" max="13" width="22"/>
+    <col bestFit="1" customWidth="1" min="14" max="14" width="16.85546875"/>
+    <col bestFit="1" customWidth="1" min="15" max="15" width="14.42578125"/>
+    <col bestFit="1" customWidth="1" min="16" max="16" width="20.42578125"/>
+    <col bestFit="1" customWidth="1" min="17" max="17" width="52"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2432,7 +2634,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -2480,7 +2682,7 @@
       </c>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -2508,7 +2710,7 @@
       <c r="I3" t="s">
         <v>28</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="3" t="s">
         <v>29</v>
       </c>
       <c r="K3" t="s">
@@ -2528,7 +2730,7 @@
       </c>
       <c r="P3" s="2"/>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -2576,7 +2778,7 @@
       </c>
       <c r="P4" s="2"/>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -2624,7 +2826,7 @@
       </c>
       <c r="P5" s="2"/>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6">
       <c r="A6" t="s">
         <v>46</v>
       </c>
@@ -2672,7 +2874,7 @@
       </c>
       <c r="P6" s="2"/>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7">
       <c r="A7" t="s">
         <v>53</v>
       </c>
@@ -2720,7 +2922,7 @@
       </c>
       <c r="P7" s="2"/>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8">
       <c r="A8" t="s">
         <v>59</v>
       </c>
@@ -2768,7 +2970,7 @@
       </c>
       <c r="P8" s="2"/>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9">
       <c r="A9" t="s">
         <v>65</v>
       </c>
@@ -2816,7 +3018,7 @@
       </c>
       <c r="P9" s="2"/>
     </row>
-    <row r="10" spans="1:17">
+    <row r="10">
       <c r="A10" t="s">
         <v>71</v>
       </c>
@@ -2864,7 +3066,7 @@
       </c>
       <c r="P10" s="2"/>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11">
       <c r="A11" t="s">
         <v>77</v>
       </c>
@@ -2912,7 +3114,7 @@
       </c>
       <c r="P11" s="2"/>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12">
       <c r="A12" t="s">
         <v>83</v>
       </c>
@@ -2960,7 +3162,7 @@
       </c>
       <c r="P12" s="2"/>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13">
       <c r="A13" t="s">
         <v>89</v>
       </c>
@@ -3008,7 +3210,7 @@
       </c>
       <c r="P13" s="2"/>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14">
       <c r="A14" t="s">
         <v>95</v>
       </c>
@@ -3056,7 +3258,7 @@
       </c>
       <c r="P14" s="2"/>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15">
       <c r="A15" t="s">
         <v>101</v>
       </c>
@@ -3104,7 +3306,7 @@
       </c>
       <c r="P15" s="2"/>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16">
       <c r="A16" t="s">
         <v>107</v>
       </c>
@@ -3152,7 +3354,7 @@
       </c>
       <c r="P16" s="2"/>
     </row>
-    <row r="17" spans="1:16">
+    <row r="17">
       <c r="A17" t="s">
         <v>113</v>
       </c>
@@ -3200,7 +3402,7 @@
       </c>
       <c r="P17" s="2"/>
     </row>
-    <row r="18" spans="1:16">
+    <row r="18">
       <c r="A18" t="s">
         <v>119</v>
       </c>
@@ -3248,7 +3450,7 @@
       </c>
       <c r="P18" s="2"/>
     </row>
-    <row r="19" spans="1:16">
+    <row r="19">
       <c r="A19" t="s">
         <v>125</v>
       </c>
@@ -3296,7 +3498,7 @@
       </c>
       <c r="P19" s="2"/>
     </row>
-    <row r="20" spans="1:16">
+    <row r="20">
       <c r="A20" t="s">
         <v>131</v>
       </c>
@@ -3344,7 +3546,7 @@
       </c>
       <c r="P20" s="2"/>
     </row>
-    <row r="21" spans="1:16">
+    <row r="21">
       <c r="A21" t="s">
         <v>137</v>
       </c>
@@ -3392,7 +3594,7 @@
       </c>
       <c r="P21" s="2"/>
     </row>
-    <row r="22" spans="1:16">
+    <row r="22">
       <c r="A22" t="s">
         <v>143</v>
       </c>
@@ -3440,7 +3642,7 @@
       </c>
       <c r="P22" s="2"/>
     </row>
-    <row r="23" spans="1:16">
+    <row r="23">
       <c r="A23" t="s">
         <v>149</v>
       </c>
@@ -3488,7 +3690,7 @@
       </c>
       <c r="P23" s="2"/>
     </row>
-    <row r="24" spans="1:16">
+    <row r="24">
       <c r="A24" t="s">
         <v>155</v>
       </c>
@@ -3536,7 +3738,7 @@
       </c>
       <c r="P24" s="2"/>
     </row>
-    <row r="25" spans="1:16">
+    <row r="25">
       <c r="A25" t="s">
         <v>161</v>
       </c>
@@ -3584,7 +3786,7 @@
       </c>
       <c r="P25" s="2"/>
     </row>
-    <row r="26" spans="1:16">
+    <row r="26">
       <c r="A26" t="s">
         <v>167</v>
       </c>
@@ -3632,7 +3834,7 @@
       </c>
       <c r="P26" s="2"/>
     </row>
-    <row r="27" spans="1:16">
+    <row r="27">
       <c r="A27" t="s">
         <v>173</v>
       </c>
@@ -3680,7 +3882,7 @@
       </c>
       <c r="P27" s="2"/>
     </row>
-    <row r="28" spans="1:16">
+    <row r="28">
       <c r="A28" t="s">
         <v>179</v>
       </c>
@@ -3728,7 +3930,7 @@
       </c>
       <c r="P28" s="2"/>
     </row>
-    <row r="29" spans="1:16">
+    <row r="29">
       <c r="A29" t="s">
         <v>185</v>
       </c>
@@ -3776,7 +3978,7 @@
       </c>
       <c r="P29" s="2"/>
     </row>
-    <row r="30" spans="1:16">
+    <row r="30">
       <c r="A30" t="s">
         <v>191</v>
       </c>
@@ -3824,7 +4026,7 @@
       </c>
       <c r="P30" s="2"/>
     </row>
-    <row r="31" spans="1:16">
+    <row r="31">
       <c r="A31" t="s">
         <v>197</v>
       </c>
@@ -3872,7 +4074,7 @@
       </c>
       <c r="P31" s="2"/>
     </row>
-    <row r="32" spans="1:16">
+    <row r="32">
       <c r="A32" t="s">
         <v>203</v>
       </c>
@@ -3920,7 +4122,7 @@
       </c>
       <c r="P32" s="2"/>
     </row>
-    <row r="33" spans="1:16">
+    <row r="33">
       <c r="A33" t="s">
         <v>209</v>
       </c>
@@ -3968,7 +4170,7 @@
       </c>
       <c r="P33" s="2"/>
     </row>
-    <row r="34" spans="1:16">
+    <row r="34">
       <c r="A34" t="s">
         <v>215</v>
       </c>
@@ -4016,7 +4218,7 @@
       </c>
       <c r="P34" s="2"/>
     </row>
-    <row r="35" spans="1:16">
+    <row r="35">
       <c r="A35" t="s">
         <v>221</v>
       </c>
@@ -4064,7 +4266,7 @@
       </c>
       <c r="P35" s="2"/>
     </row>
-    <row r="36" spans="1:16">
+    <row r="36">
       <c r="A36" t="s">
         <v>227</v>
       </c>
@@ -4112,7 +4314,7 @@
       </c>
       <c r="P36" s="2"/>
     </row>
-    <row r="37" spans="1:16">
+    <row r="37">
       <c r="A37" t="s">
         <v>233</v>
       </c>
@@ -4160,7 +4362,7 @@
       </c>
       <c r="P37" s="2"/>
     </row>
-    <row r="38" spans="1:16">
+    <row r="38">
       <c r="A38" t="s">
         <v>239</v>
       </c>
@@ -4208,7 +4410,7 @@
       </c>
       <c r="P38" s="2"/>
     </row>
-    <row r="39" spans="1:16">
+    <row r="39">
       <c r="A39" t="s">
         <v>245</v>
       </c>
@@ -4256,7 +4458,7 @@
       </c>
       <c r="P39" s="2"/>
     </row>
-    <row r="40" spans="1:16">
+    <row r="40">
       <c r="A40" t="s">
         <v>251</v>
       </c>
@@ -4304,7 +4506,7 @@
       </c>
       <c r="P40" s="2"/>
     </row>
-    <row r="41" spans="1:16">
+    <row r="41">
       <c r="A41" t="s">
         <v>257</v>
       </c>
@@ -4352,7 +4554,7 @@
       </c>
       <c r="P41" s="2"/>
     </row>
-    <row r="42" spans="1:16">
+    <row r="42">
       <c r="A42" t="s">
         <v>263</v>
       </c>
@@ -4400,7 +4602,7 @@
       </c>
       <c r="P42" s="2"/>
     </row>
-    <row r="43" spans="1:16">
+    <row r="43">
       <c r="A43" t="s">
         <v>269</v>
       </c>
@@ -4448,7 +4650,7 @@
       </c>
       <c r="P43" s="2"/>
     </row>
-    <row r="44" spans="1:16">
+    <row r="44">
       <c r="A44" t="s">
         <v>275</v>
       </c>
@@ -4496,7 +4698,7 @@
       </c>
       <c r="P44" s="2"/>
     </row>
-    <row r="45" spans="1:16">
+    <row r="45">
       <c r="A45" t="s">
         <v>281</v>
       </c>
@@ -4544,7 +4746,7 @@
       </c>
       <c r="P45" s="2"/>
     </row>
-    <row r="46" spans="1:16">
+    <row r="46">
       <c r="A46" t="s">
         <v>287</v>
       </c>
@@ -4592,7 +4794,7 @@
       </c>
       <c r="P46" s="2"/>
     </row>
-    <row r="47" spans="1:16">
+    <row r="47">
       <c r="A47" t="s">
         <v>293</v>
       </c>
@@ -4640,7 +4842,7 @@
       </c>
       <c r="P47" s="2"/>
     </row>
-    <row r="48" spans="1:16">
+    <row r="48">
       <c r="A48" t="s">
         <v>299</v>
       </c>
@@ -4688,7 +4890,7 @@
       </c>
       <c r="P48" s="2"/>
     </row>
-    <row r="49" spans="1:16">
+    <row r="49">
       <c r="A49" t="s">
         <v>305</v>
       </c>
@@ -4736,7 +4938,7 @@
       </c>
       <c r="P49" s="2"/>
     </row>
-    <row r="50" spans="1:16">
+    <row r="50">
       <c r="A50" t="s">
         <v>311</v>
       </c>
@@ -4784,7 +4986,7 @@
       </c>
       <c r="P50" s="2"/>
     </row>
-    <row r="51" spans="1:16">
+    <row r="51">
       <c r="A51" t="s">
         <v>317</v>
       </c>
@@ -4832,7 +5034,7 @@
       </c>
       <c r="P51" s="2"/>
     </row>
-    <row r="52" spans="1:16">
+    <row r="52">
       <c r="A52" t="s">
         <v>323</v>
       </c>
@@ -4880,7 +5082,7 @@
       </c>
       <c r="P52" s="2"/>
     </row>
-    <row r="53" spans="1:16">
+    <row r="53">
       <c r="A53" t="s">
         <v>329</v>
       </c>
@@ -4928,7 +5130,7 @@
       </c>
       <c r="P53" s="2"/>
     </row>
-    <row r="54" spans="1:16">
+    <row r="54">
       <c r="A54" t="s">
         <v>335</v>
       </c>
@@ -4976,7 +5178,7 @@
       </c>
       <c r="P54" s="2"/>
     </row>
-    <row r="55" spans="1:16">
+    <row r="55">
       <c r="A55" t="s">
         <v>341</v>
       </c>
@@ -5024,7 +5226,7 @@
       </c>
       <c r="P55" s="2"/>
     </row>
-    <row r="56" spans="1:16">
+    <row r="56">
       <c r="A56" t="s">
         <v>347</v>
       </c>
@@ -5072,7 +5274,7 @@
       </c>
       <c r="P56" s="2"/>
     </row>
-    <row r="57" spans="1:16">
+    <row r="57">
       <c r="A57" t="s">
         <v>353</v>
       </c>
@@ -5120,7 +5322,7 @@
       </c>
       <c r="P57" s="2"/>
     </row>
-    <row r="58" spans="1:16">
+    <row r="58">
       <c r="A58" t="s">
         <v>359</v>
       </c>
@@ -5168,7 +5370,7 @@
       </c>
       <c r="P58" s="2"/>
     </row>
-    <row r="59" spans="1:16">
+    <row r="59">
       <c r="A59" t="s">
         <v>365</v>
       </c>
@@ -5216,7 +5418,7 @@
       </c>
       <c r="P59" s="2"/>
     </row>
-    <row r="60" spans="1:16">
+    <row r="60">
       <c r="A60" t="s">
         <v>371</v>
       </c>
@@ -5264,7 +5466,7 @@
       </c>
       <c r="P60" s="2"/>
     </row>
-    <row r="61" spans="1:16">
+    <row r="61">
       <c r="A61" t="s">
         <v>377</v>
       </c>
@@ -5312,7 +5514,7 @@
       </c>
       <c r="P61" s="2"/>
     </row>
-    <row r="62" spans="1:16">
+    <row r="62">
       <c r="A62" t="s">
         <v>383</v>
       </c>
@@ -5360,7 +5562,7 @@
       </c>
       <c r="P62" s="2"/>
     </row>
-    <row r="63" spans="1:16">
+    <row r="63">
       <c r="A63" t="s">
         <v>389</v>
       </c>
@@ -5408,7 +5610,7 @@
       </c>
       <c r="P63" s="2"/>
     </row>
-    <row r="64" spans="1:16">
+    <row r="64">
       <c r="A64" t="s">
         <v>395</v>
       </c>
@@ -5456,7 +5658,7 @@
       </c>
       <c r="P64" s="2"/>
     </row>
-    <row r="65" spans="1:16">
+    <row r="65">
       <c r="A65" t="s">
         <v>401</v>
       </c>
@@ -5504,7 +5706,7 @@
       </c>
       <c r="P65" s="2"/>
     </row>
-    <row r="66" spans="1:16">
+    <row r="66">
       <c r="A66" t="s">
         <v>407</v>
       </c>
@@ -5552,7 +5754,7 @@
       </c>
       <c r="P66" s="2"/>
     </row>
-    <row r="67" spans="1:16">
+    <row r="67">
       <c r="A67" t="s">
         <v>413</v>
       </c>
@@ -5600,7 +5802,7 @@
       </c>
       <c r="P67" s="2"/>
     </row>
-    <row r="68" spans="1:16">
+    <row r="68">
       <c r="A68" t="s">
         <v>419</v>
       </c>
@@ -5648,7 +5850,7 @@
       </c>
       <c r="P68" s="2"/>
     </row>
-    <row r="69" spans="1:16">
+    <row r="69">
       <c r="A69" t="s">
         <v>425</v>
       </c>
@@ -5696,7 +5898,7 @@
       </c>
       <c r="P69" s="2"/>
     </row>
-    <row r="70" spans="1:16">
+    <row r="70">
       <c r="A70" t="s">
         <v>431</v>
       </c>
@@ -5744,7 +5946,7 @@
       </c>
       <c r="P70" s="2"/>
     </row>
-    <row r="71" spans="1:16">
+    <row r="71">
       <c r="A71" t="s">
         <v>437</v>
       </c>
@@ -5792,7 +5994,7 @@
       </c>
       <c r="P71" s="2"/>
     </row>
-    <row r="72" spans="1:16">
+    <row r="72">
       <c r="A72" t="s">
         <v>443</v>
       </c>
@@ -5840,7 +6042,7 @@
       </c>
       <c r="P72" s="2"/>
     </row>
-    <row r="73" spans="1:16">
+    <row r="73">
       <c r="A73" t="s">
         <v>449</v>
       </c>
@@ -5888,7 +6090,7 @@
       </c>
       <c r="P73" s="2"/>
     </row>
-    <row r="74" spans="1:16">
+    <row r="74">
       <c r="A74" t="s">
         <v>455</v>
       </c>
@@ -5936,7 +6138,7 @@
       </c>
       <c r="P74" s="2"/>
     </row>
-    <row r="75" spans="1:16">
+    <row r="75">
       <c r="A75" t="s">
         <v>461</v>
       </c>
@@ -5984,7 +6186,7 @@
       </c>
       <c r="P75" s="2"/>
     </row>
-    <row r="76" spans="1:16">
+    <row r="76">
       <c r="A76" t="s">
         <v>467</v>
       </c>
@@ -6032,7 +6234,7 @@
       </c>
       <c r="P76" s="2"/>
     </row>
-    <row r="77" spans="1:16">
+    <row r="77">
       <c r="A77" t="s">
         <v>473</v>
       </c>
@@ -6080,7 +6282,7 @@
       </c>
       <c r="P77" s="2"/>
     </row>
-    <row r="78" spans="1:16">
+    <row r="78">
       <c r="A78" t="s">
         <v>479</v>
       </c>
@@ -6128,7 +6330,7 @@
       </c>
       <c r="P78" s="2"/>
     </row>
-    <row r="79" spans="1:16">
+    <row r="79">
       <c r="A79" t="s">
         <v>485</v>
       </c>
@@ -6176,7 +6378,7 @@
       </c>
       <c r="P79" s="2"/>
     </row>
-    <row r="80" spans="1:16">
+    <row r="80">
       <c r="A80" t="s">
         <v>491</v>
       </c>
@@ -6224,7 +6426,7 @@
       </c>
       <c r="P80" s="2"/>
     </row>
-    <row r="81" spans="1:16">
+    <row r="81">
       <c r="A81" t="s">
         <v>497</v>
       </c>
@@ -6272,7 +6474,7 @@
       </c>
       <c r="P81" s="2"/>
     </row>
-    <row r="82" spans="1:16">
+    <row r="82">
       <c r="A82" t="s">
         <v>503</v>
       </c>
@@ -6320,7 +6522,7 @@
       </c>
       <c r="P82" s="2"/>
     </row>
-    <row r="83" spans="1:16">
+    <row r="83">
       <c r="A83" t="s">
         <v>509</v>
       </c>
@@ -6368,7 +6570,7 @@
       </c>
       <c r="P83" s="2"/>
     </row>
-    <row r="84" spans="1:16">
+    <row r="84">
       <c r="A84" t="s">
         <v>515</v>
       </c>
@@ -6416,7 +6618,7 @@
       </c>
       <c r="P84" s="2"/>
     </row>
-    <row r="85" spans="1:16">
+    <row r="85">
       <c r="A85" t="s">
         <v>521</v>
       </c>
@@ -6464,7 +6666,7 @@
       </c>
       <c r="P85" s="2"/>
     </row>
-    <row r="86" spans="1:16">
+    <row r="86">
       <c r="A86" t="s">
         <v>527</v>
       </c>
@@ -6512,7 +6714,7 @@
       </c>
       <c r="P86" s="2"/>
     </row>
-    <row r="87" spans="1:16">
+    <row r="87">
       <c r="A87" t="s">
         <v>533</v>
       </c>
@@ -6560,7 +6762,7 @@
       </c>
       <c r="P87" s="2"/>
     </row>
-    <row r="88" spans="1:16">
+    <row r="88">
       <c r="A88" t="s">
         <v>539</v>
       </c>
@@ -6608,7 +6810,7 @@
       </c>
       <c r="P88" s="2"/>
     </row>
-    <row r="89" spans="1:16">
+    <row r="89">
       <c r="A89" t="s">
         <v>545</v>
       </c>
@@ -6656,7 +6858,7 @@
       </c>
       <c r="P89" s="2"/>
     </row>
-    <row r="90" spans="1:16">
+    <row r="90">
       <c r="A90" t="s">
         <v>551</v>
       </c>
@@ -6704,7 +6906,7 @@
       </c>
       <c r="P90" s="2"/>
     </row>
-    <row r="91" spans="1:16">
+    <row r="91">
       <c r="A91" t="s">
         <v>557</v>
       </c>
@@ -6752,7 +6954,7 @@
       </c>
       <c r="P91" s="2"/>
     </row>
-    <row r="92" spans="1:16">
+    <row r="92">
       <c r="A92" t="s">
         <v>563</v>
       </c>
@@ -6800,7 +7002,7 @@
       </c>
       <c r="P92" s="2"/>
     </row>
-    <row r="93" spans="1:16">
+    <row r="93">
       <c r="A93" t="s">
         <v>569</v>
       </c>
@@ -6848,7 +7050,7 @@
       </c>
       <c r="P93" s="2"/>
     </row>
-    <row r="94" spans="1:16">
+    <row r="94">
       <c r="A94" t="s">
         <v>575</v>
       </c>
@@ -6896,7 +7098,7 @@
       </c>
       <c r="P94" s="2"/>
     </row>
-    <row r="95" spans="1:16">
+    <row r="95">
       <c r="A95" t="s">
         <v>581</v>
       </c>
@@ -6944,7 +7146,7 @@
       </c>
       <c r="P95" s="2"/>
     </row>
-    <row r="96" spans="1:16">
+    <row r="96">
       <c r="A96" t="s">
         <v>587</v>
       </c>
@@ -6992,7 +7194,7 @@
       </c>
       <c r="P96" s="2"/>
     </row>
-    <row r="97" spans="1:16">
+    <row r="97">
       <c r="A97" t="s">
         <v>593</v>
       </c>
@@ -7040,7 +7242,7 @@
       </c>
       <c r="P97" s="2"/>
     </row>
-    <row r="98" spans="1:16">
+    <row r="98">
       <c r="A98" t="s">
         <v>599</v>
       </c>
@@ -7088,7 +7290,7 @@
       </c>
       <c r="P98" s="2"/>
     </row>
-    <row r="99" spans="1:16">
+    <row r="99">
       <c r="A99" t="s">
         <v>605</v>
       </c>
@@ -7136,7 +7338,7 @@
       </c>
       <c r="P99" s="2"/>
     </row>
-    <row r="100" spans="1:16">
+    <row r="100">
       <c r="A100" t="s">
         <v>611</v>
       </c>
@@ -7184,7 +7386,7 @@
       </c>
       <c r="P100" s="2"/>
     </row>
-    <row r="101" spans="1:16">
+    <row r="101">
       <c r="A101" t="s">
         <v>617</v>
       </c>
@@ -7233,7 +7435,13 @@
       <c r="P101" s="2"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="J3"/>
+  </hyperlinks>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
@@ -7375,9 +7583,7 @@
         <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
         <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
           <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
+            <xsd:documentation>This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.</xsd:documentation>
           </xsd:annotation>
         </xsd:element>
         <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -7465,13 +7671,41 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ED20BC1-588F-4C67-9125-374558E08EB6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="1ed20bc1-588f-4c67-9125-374558e08eb6">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema-instance"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cceef600-efdf-45e2-9e7c-b2c141a53b00"/>
+    <ds:schemaRef ds:uri="e06cef04-58b7-49df-a0f0-ed4b003b0a7f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AA55681-4EBF-400B-8EEB-966CF134C9AE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="7aa55681-4ebf-400b-8eeb-966cf134c9ae">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="cceef600-efdf-45e2-9e7c-b2c141a53b00"/>
+    <ds:schemaRef ds:uri="e06cef04-58b7-49df-a0f0-ed4b003b0a7f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema-instance"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1C14E08-09F8-4EE0-8656-4DA5E95E5EC4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="b1c14e08-09f8-4ee0-8656-4da5e95e5ec4">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>